<commit_message>
feat: complete AI document scanner, email reply identity, contact UI and potential customer assigned sale
</commit_message>
<xml_diff>
--- a/Web/public/mau-import-tin-dang.xlsx
+++ b/Web/public/mau-import-tin-dang.xlsx
@@ -1,58 +1,241 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Tin đăng" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Danh sách tin đăng" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Hướng dẫn điền dữ liệu" state="visible" r:id="rId5"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
+  <si>
+    <t>Tiêu đề tin (*)</t>
+  </si>
+  <si>
+    <t>Mức giá (*)</t>
+  </si>
+  <si>
+    <t>Vị trí / Địa chỉ (*)</t>
+  </si>
+  <si>
+    <t>Diện tích (m2)</t>
+  </si>
+  <si>
+    <t>Số phòng ngủ</t>
+  </si>
+  <si>
+    <t>Số phòng tắm</t>
+  </si>
+  <si>
+    <t>Hình thức</t>
+  </si>
+  <si>
+    <t>Loại BĐS</t>
+  </si>
+  <si>
+    <t>Pháp lý</t>
+  </si>
+  <si>
+    <t>Mô tả chi tiết</t>
+  </si>
+  <si>
+    <t>Hình ảnh URL</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
+    <t>Bán căn hộ 2 phòng ngủ view biển Lộc Thọ</t>
+  </si>
+  <si>
+    <t>2.85 tỷ</t>
+  </si>
+  <si>
+    <t>Lộc Thọ, Nha Trang</t>
+  </si>
+  <si>
+    <t>Bán</t>
+  </si>
+  <si>
+    <t>Căn hộ</t>
+  </si>
+  <si>
+    <t>Sổ hồng lâu dài</t>
+  </si>
+  <si>
+    <t>Căn hộ tầng cao thoáng mát, view biển trực diện, đầy đủ nội thất cao cấp.</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1545324418-cc1a3fa10c00?w=800</t>
+  </si>
+  <si>
+    <t>Đã duyệt</t>
+  </si>
+  <si>
+    <t>Cho thuê nhà phố 3 tầng trung tâm Phước Hải</t>
+  </si>
+  <si>
+    <t>15 triệu/tháng</t>
+  </si>
+  <si>
+    <t>Phước Hải, Nha Trang</t>
+  </si>
+  <si>
+    <t>Cho thuê</t>
+  </si>
+  <si>
+    <t>Nhà phố</t>
+  </si>
+  <si>
+    <t>Sổ đỏ chính chủ</t>
+  </si>
+  <si>
+    <t>Nhà phố mặt tiền đường lớn, tiện kinh doanh buôn bán hoặc mở văn phòng công ty.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Chờ duyệt</t>
+  </si>
+  <si>
+    <t>Bán đất nền thổ cư Diên Khánh giá tốt</t>
+  </si>
+  <si>
+    <t>1.5 tỷ</t>
+  </si>
+  <si>
+    <t>Diên Khánh, Khánh Hòa</t>
+  </si>
+  <si>
+    <t>Đất nền</t>
+  </si>
+  <si>
+    <t>Sổ đỏ riêng</t>
+  </si>
+  <si>
+    <t>Đất vuông vức, đường bê tông 6m ô tô quay đầu, điện nước đầy đủ, xây dựng ngay.</t>
+  </si>
+  <si>
+    <t>Tên cột</t>
+  </si>
+  <si>
+    <t>Bắt buộc</t>
+  </si>
+  <si>
+    <t>Quy tắc / Định dạng</t>
+  </si>
+  <si>
+    <t>Ví dụ hợp lệ</t>
+  </si>
+  <si>
+    <t>BẮT BUỘC</t>
+  </si>
+  <si>
+    <t>Tên tin đăng rõ ràng, không để trống</t>
+  </si>
+  <si>
+    <t>Bán căn hộ 2PN Masteri view sông</t>
+  </si>
+  <si>
+    <t>Ghi rõ số tiền kèm đơn vị (tỷ, triệu, triệu/tháng)</t>
+  </si>
+  <si>
+    <t>3.2 tỷ hoặc 15 triệu/tháng</t>
+  </si>
+  <si>
+    <t>Quận/Huyện, Tỉnh/TP hoặc tên dự án</t>
+  </si>
+  <si>
+    <t>Quận 2, TP.HCM hoặc Lộc Thọ, Nha Trang</t>
+  </si>
+  <si>
+    <t>Tùy chọn</t>
+  </si>
+  <si>
+    <t>Số nguyên hoặc số thập phân</t>
+  </si>
+  <si>
+    <t>75 hoặc 85.5</t>
+  </si>
+  <si>
+    <t>Số nguyên (1, 2, 3...)</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Chọn dạng thả xuống: Bán hoặc Cho thuê</t>
+  </si>
+  <si>
+    <t>Chọn dạng thả xuống: Căn hộ, Nhà phố, Biệt thự, Đất nền, Shophouse</t>
+  </si>
+  <si>
+    <t>Sổ hồng, Sổ đỏ chính chủ, Hợp đồng mua bán...</t>
+  </si>
+  <si>
+    <t>Nội dung mô tả thêm về tiện ích, kết cấu...</t>
+  </si>
+  <si>
+    <t>Căn góc, view thoáng, nội thất cơ bản</t>
+  </si>
+  <si>
+    <t>Đường dẫn ảnh trực tiếp (http/https)</t>
+  </si>
+  <si>
+    <t>https://example.com/anh.jpg</t>
+  </si>
+  <si>
+    <t>Chọn dạng thả xuống: Chờ duyệt hoặc Đã duyệt (Mặc định: Chờ duyệt)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFDC2626"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F2A44"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +243,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0D5C56"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF0D5C56"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0D5C56"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF0B4A45"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,56 +609,70 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L200"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="45" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>title</v>
-      </c>
-      <c r="B1" t="str">
-        <v>price</v>
-      </c>
-      <c r="C1" t="str">
-        <v>location</v>
-      </c>
-      <c r="D1" t="str">
-        <v>area</v>
-      </c>
-      <c r="E1" t="str">
-        <v>beds</v>
-      </c>
-      <c r="F1" t="str">
-        <v>baths</v>
-      </c>
-      <c r="G1" t="str">
-        <v>transactionType</v>
-      </c>
-      <c r="H1" t="str">
-        <v>propertyType</v>
-      </c>
-      <c r="I1" t="str">
-        <v>legalStatus</v>
-      </c>
-      <c r="J1" t="str">
-        <v>description</v>
-      </c>
-      <c r="K1" t="str">
-        <v>imageUrl</v>
-      </c>
-      <c r="L1" t="str">
-        <v>status</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Bán căn hộ mẫu tại Nha Trang</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2.5 tỷ</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Lộc Thọ, Nha Trang</v>
+    <row r="1" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
       </c>
       <c r="D2">
         <v>75</v>
@@ -456,34 +683,34 @@
       <c r="F2">
         <v>2</v>
       </c>
-      <c r="G2" t="str">
-        <v>sale</v>
-      </c>
-      <c r="H2" t="str">
-        <v>apartment</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Sổ hồng</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Tin mẫu để kiểm tra import Excel.</v>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Cho thuê nhà phố mẫu</v>
-      </c>
-      <c r="B3" t="str">
-        <v>12 triệu/tháng</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Phước Hải, Nha Trang</v>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
       </c>
       <c r="D3">
         <v>100</v>
@@ -492,30 +719,476 @@
         <v>3</v>
       </c>
       <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="9" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="11" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="13" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="14" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="15" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="16" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="17" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="19" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="20" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="21" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="22" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="25" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="26" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="27" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="29" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="30" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="32" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="33" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="35" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="36" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="37" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="39" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="40" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="41" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="42" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="43" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="44" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="45" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="46" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="48" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="49" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="51" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="52" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="53" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="54" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="55" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="56" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="57" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="58" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="59" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="60" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="61" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="62" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="63" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="64" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="76" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="77" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="79" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="80" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="134" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="135" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="137" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="138" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="139" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="140" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="141" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="142" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="143" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="144" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="149" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="150" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="151" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="152" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="153" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="154" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="155" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="156" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="157" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="158" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="159" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="160" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="22" customHeight="1" spans="7:12" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn hình thức không hợp lệ" error="Vui lòng chọn từ danh sách: Bán hoặc Cho thuê" sqref="G10:G200">
+      <formula1>"Bán,Cho thuê"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn hình thức không hợp lệ" error="Vui lòng chọn từ danh sách: Bán hoặc Cho thuê" sqref="G2:G200">
+      <formula1>"Bán,Cho thuê"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn loại BĐS không hợp lệ" error="Vui lòng chọn từ danh sách: Căn hộ, Nhà phố, Biệt thự, Đất nền, hoặc Shophouse" sqref="H10:H200">
+      <formula1>"Căn hộ,Nhà phố,Biệt thự,Đất nền,Shophouse"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn loại BĐS không hợp lệ" error="Vui lòng chọn từ danh sách: Căn hộ, Nhà phố, Biệt thự, Đất nền, hoặc Shophouse" sqref="H2:H200">
+      <formula1>"Căn hộ,Nhà phố,Biệt thự,Đất nền,Shophouse"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn trạng thái không hợp lệ" error="Vui lòng chọn từ danh sách: Chờ duyệt hoặc Đã duyệt" sqref="L10:L200">
+      <formula1>"Chờ duyệt,Đã duyệt"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Chọn trạng thái không hợp lệ" error="Vui lòng chọn từ danh sách: Chờ duyệt hoặc Đã duyệt" sqref="L2:L200">
+      <formula1>"Chờ duyệt,Đã duyệt"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="35" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="G3" t="str">
-        <v>rent</v>
-      </c>
-      <c r="H3" t="str">
-        <v>townhouse</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Sổ hồng</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Tin mẫu thứ hai.</v>
-      </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
-        <v>Pending</v>
+      <c r="B4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>